<commit_message>
chore: atualizacao SICARD 2026-10-28 19:37
</commit_message>
<xml_diff>
--- a/documentacao/matrizes/Matriz_PLI_v6_Blocos_Dimensoes.xlsx
+++ b/documentacao/matrizes/Matriz_PLI_v6_Blocos_Dimensoes.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dimensões de Critérios'!$A$1:$C$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Critérios'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Matriz Crit Premissas v3'!$A$1:$N$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Notas de preenchimento'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Notas de preenchimento'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rastreabilidade PLI'!$A$1:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fonte PLI v6'!$A$1:$B$156</definedName>
   </definedNames>
@@ -874,7 +874,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Bloco original do PLI. Abrange: D1 · Técnica e logística | D2 · Econômica. Fonte: PLI_Fig_Estrutura_Criterios_v6.pptx, slide 1.</t>
+          <t>Bloco original do PLI. Abrange: D1 · Eficiência logística | D2 · Econômica. Fonte: PLI_Fig_Estrutura_Criterios_v6.pptx, slide 1.</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>D1 · Técnica e logística</t>
+          <t>D1 · Eficiência logística</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>D1 · Técnica e logística</t>
+          <t>D1 · Eficiência logística</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Avaliar a dimensão D1 · Técnica e logística por meio dos indicadores T1 · Saturação e alívio de gargalos | T2 · Tempo e confiabilidade | T3 · Conectividade e intermodalidade. Objetivos associados: OE6 OE5 (em validação). O documento apresenta a hierarquia, mas não define a regra de síntese dos indicadores em uma nota da dimensão nem seus pesos. Nesta matriz, a dimensão original constitui um critério; seus indicadores são referências de composição, não critérios adicionais. O critério considera somente os componentes da fase indicada.</t>
+          <t>Avaliar a dimensão D1 · Eficiência logística por meio dos indicadores T1 · Saturação e alívio de gargalos | T2 · Tempo e confiabilidade | T3 · Conectividade e intermodalidade. Objetivos associados: OE6 OE5 (em validação). O documento apresenta a hierarquia, mas não define a regra de síntese dos indicadores em uma nota da dimensão nem seus pesos. Nesta matriz, a dimensão original constitui um critério; seus indicadores são referências de composição, não critérios adicionais. O critério considera somente os componentes da fase indicada.</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1932,17 +1932,29 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
+          <t>Nomenclatura D1</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Por solicitação do usuário, D1 · Técnica e logística passa a D1 · Eficiência logística nos campos operacionais. O nome original permanece nas abas Fonte PLI v6 e Rastreabilidade PLI. Fases, indicadores e regras não foram alterados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
           <t>Transcrição</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>A aba Fonte PLI v6 transcreve todos os textos dos dois slides, incluindo a meta e os objetivos estratégicos. Não foram utilizadas fontes normativas externas.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B20"/>
+  <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>